<commit_message>
Deploy: Content update from main workspace 2026-07-09 22:15
</commit_message>
<xml_diff>
--- a/public/blog-13-xlsx.xlsx
+++ b/public/blog-13-xlsx.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="subtitles" sheetId="1" r:id="R09d26eec39f04028"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="subtitles" sheetId="1" r:id="R66c6f4fdb8424845"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -158,9 +158,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -305,9 +305,7 @@
       <x:c r="D2" s="16" t="str">
         <x:v>en</x:v>
       </x:c>
-      <x:c r="E2" s="16" t="str">
-        <x:v>Surtitles</x:v>
-      </x:c>
+      <x:c r="E2" s="16"/>
       <x:c r="F2" s="16" t="str">
         <x:v>center</x:v>
       </x:c>
@@ -325,9 +323,7 @@
       <x:c r="D3" s="16" t="str">
         <x:v>en</x:v>
       </x:c>
-      <x:c r="E3" s="16" t="str">
-        <x:v>Surtitles</x:v>
-      </x:c>
+      <x:c r="E3" s="16"/>
       <x:c r="F3" s="16" t="str">
         <x:v>center</x:v>
       </x:c>
@@ -345,9 +341,7 @@
       <x:c r="D4" s="16" t="str">
         <x:v>en</x:v>
       </x:c>
-      <x:c r="E4" s="16" t="str">
-        <x:v>Surtitles</x:v>
-      </x:c>
+      <x:c r="E4" s="16"/>
       <x:c r="F4" s="16" t="str">
         <x:v>center</x:v>
       </x:c>
@@ -365,9 +359,7 @@
       <x:c r="D5" s="16" t="str">
         <x:v>en</x:v>
       </x:c>
-      <x:c r="E5" s="16" t="str">
-        <x:v>Surtitles</x:v>
-      </x:c>
+      <x:c r="E5" s="16"/>
       <x:c r="F5" s="16" t="str">
         <x:v>center</x:v>
       </x:c>
@@ -385,9 +377,7 @@
       <x:c r="D6" s="16" t="str">
         <x:v>en</x:v>
       </x:c>
-      <x:c r="E6" s="16" t="str">
-        <x:v>Surtitles</x:v>
-      </x:c>
+      <x:c r="E6" s="16"/>
       <x:c r="F6" s="16" t="str">
         <x:v>center</x:v>
       </x:c>
@@ -405,9 +395,7 @@
       <x:c r="D7" s="16" t="str">
         <x:v>en</x:v>
       </x:c>
-      <x:c r="E7" s="16" t="str">
-        <x:v>Surtitles</x:v>
-      </x:c>
+      <x:c r="E7" s="16"/>
       <x:c r="F7" s="16" t="str">
         <x:v>center</x:v>
       </x:c>
@@ -425,9 +413,7 @@
       <x:c r="D8" s="16" t="str">
         <x:v>en</x:v>
       </x:c>
-      <x:c r="E8" s="16" t="str">
-        <x:v>Surtitles</x:v>
-      </x:c>
+      <x:c r="E8" s="16"/>
       <x:c r="F8" s="16" t="str">
         <x:v>center</x:v>
       </x:c>
@@ -445,9 +431,7 @@
       <x:c r="D9" s="16" t="str">
         <x:v>en</x:v>
       </x:c>
-      <x:c r="E9" s="16" t="str">
-        <x:v>Surtitles</x:v>
-      </x:c>
+      <x:c r="E9" s="16"/>
       <x:c r="F9" s="16" t="str">
         <x:v>center</x:v>
       </x:c>
@@ -465,9 +449,7 @@
       <x:c r="D10" s="16" t="str">
         <x:v>en</x:v>
       </x:c>
-      <x:c r="E10" s="16" t="str">
-        <x:v>Surtitles</x:v>
-      </x:c>
+      <x:c r="E10" s="16"/>
       <x:c r="F10" s="16" t="str">
         <x:v>center</x:v>
       </x:c>
@@ -485,9 +467,7 @@
       <x:c r="D11" s="16" t="str">
         <x:v>en</x:v>
       </x:c>
-      <x:c r="E11" s="16" t="str">
-        <x:v>Surtitles</x:v>
-      </x:c>
+      <x:c r="E11" s="16"/>
       <x:c r="F11" s="16" t="str">
         <x:v>center</x:v>
       </x:c>
@@ -505,9 +485,7 @@
       <x:c r="D12" s="16" t="str">
         <x:v>en</x:v>
       </x:c>
-      <x:c r="E12" s="16" t="str">
-        <x:v>Surtitles</x:v>
-      </x:c>
+      <x:c r="E12" s="16"/>
       <x:c r="F12" s="16" t="str">
         <x:v>center</x:v>
       </x:c>
@@ -525,9 +503,7 @@
       <x:c r="D13" s="16" t="str">
         <x:v>en</x:v>
       </x:c>
-      <x:c r="E13" s="16" t="str">
-        <x:v>Surtitles</x:v>
-      </x:c>
+      <x:c r="E13" s="16"/>
       <x:c r="F13" s="16" t="str">
         <x:v>center</x:v>
       </x:c>
@@ -546,7 +522,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4297ba7be98043a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbad15c02e95b4c5e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>